<commit_message>
feat(ag): add workflow for PGV dossiers
</commit_message>
<xml_diff>
--- a/django/kt_ag/import/Services_AG.xlsx
+++ b/django/kt_ag/import/Services_AG.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="113">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -356,6 +356,9 @@
   </si>
   <si>
     <t xml:space="preserve">gemeindeverwaltung@zuzgen.ch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leitbehörde PGV</t>
   </si>
 </sst>
 </file>
@@ -670,10 +673,10 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="86.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="86.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.85"/>
@@ -1722,6 +1725,17 @@
       </c>
       <c r="J79" s="1" t="n">
         <v>4264</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="I80" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
chore(ag): remove two services from import file
</commit_message>
<xml_diff>
--- a/django/kt_ag/import/Services_AG.xlsx
+++ b/django/kt_ag/import/Services_AG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$K$264</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$K$262</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="319">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -275,15 +275,6 @@
   </si>
   <si>
     <t xml:space="preserve">Eidgenössischer Schiessoffizier (ESO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eidgenössiches Starkstorminspektorat (ESTI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gasverbund Mittelland AG (GVM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gvm</t>
   </si>
   <si>
     <t xml:space="preserve">SBB</t>
@@ -1102,36 +1093,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1363,8 +1358,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K264"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K1048576"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="86.25"/>
@@ -1917,8 +1912,8 @@
       <c r="B42" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
       <c r="J42" s="1" t="n">
         <v>0</v>
       </c>
@@ -2052,11 +2047,8 @@
       <c r="A53" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="J53" s="1" t="n">
         <v>0</v>
@@ -2067,7 +2059,25 @@
         <v>4</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>87</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>4600</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H54" s="1" t="n">
+        <v>622068850</v>
       </c>
       <c r="J54" s="1" t="n">
         <v>0</v>
@@ -2075,10 +2085,13 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="J55" s="1" t="n">
         <v>0</v>
@@ -2086,76 +2099,64 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E56" s="1" t="n">
-        <v>4600</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H56" s="1" t="n">
-        <v>622068850</v>
+        <v>14</v>
       </c>
       <c r="J56" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>4001</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="J57" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>4271</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>14</v>
+        <v>95</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="J58" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K58" s="1" t="n">
-        <v>4001</v>
+        <v>4221</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D59" s="1" t="s">
         <v>97</v>
       </c>
       <c r="J59" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K59" s="1" t="n">
-        <v>4271</v>
+        <v>4191</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2165,28 +2166,28 @@
       <c r="B60" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D60" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="J60" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K60" s="1" t="n">
-        <v>4221</v>
+        <v>4222</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>100</v>
       </c>
       <c r="J61" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K61" s="1" t="n">
-        <v>4191</v>
+        <v>4061</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2200,24 +2201,21 @@
         <v>0</v>
       </c>
       <c r="K62" s="1" t="n">
-        <v>4222</v>
+        <v>4091</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D63" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="J63" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K63" s="1" t="n">
-        <v>4061</v>
+        <v>4223</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2225,13 +2223,13 @@
         <v>6</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J64" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K64" s="1" t="n">
-        <v>4091</v>
+        <v>4021</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2239,13 +2237,13 @@
         <v>6</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J65" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K65" s="1" t="n">
-        <v>4223</v>
+        <v>4224</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2253,13 +2251,13 @@
         <v>6</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J66" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K66" s="1" t="n">
-        <v>4021</v>
+        <v>4131</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2267,13 +2265,13 @@
         <v>6</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J67" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K67" s="1" t="n">
-        <v>4224</v>
+        <v>4022</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2281,13 +2279,13 @@
         <v>6</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J68" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K68" s="1" t="n">
-        <v>4131</v>
+        <v>4023</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2295,13 +2293,13 @@
         <v>6</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J69" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K69" s="1" t="n">
-        <v>4022</v>
+        <v>4062</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2309,13 +2307,13 @@
         <v>6</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J70" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K70" s="1" t="n">
-        <v>4023</v>
+        <v>4226</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2323,27 +2321,30 @@
         <v>6</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J71" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K71" s="1" t="n">
-        <v>4062</v>
+        <v>4227</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>112</v>
       </c>
       <c r="J72" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K72" s="1" t="n">
-        <v>4226</v>
+        <v>4002</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2357,24 +2358,21 @@
         <v>0</v>
       </c>
       <c r="K73" s="1" t="n">
-        <v>4227</v>
+        <v>4024</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D74" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="J74" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K74" s="1" t="n">
-        <v>4002</v>
+        <v>4092</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2382,13 +2380,13 @@
         <v>6</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J75" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K75" s="1" t="n">
-        <v>4024</v>
+        <v>4093</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,13 +2394,13 @@
         <v>6</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J76" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K76" s="1" t="n">
-        <v>4092</v>
+        <v>4132</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2410,13 +2408,13 @@
         <v>6</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J77" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K77" s="1" t="n">
-        <v>4093</v>
+        <v>4192</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2424,13 +2422,13 @@
         <v>6</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J78" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K78" s="1" t="n">
-        <v>4132</v>
+        <v>4228</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2438,13 +2436,13 @@
         <v>6</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J79" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K79" s="1" t="n">
-        <v>4192</v>
+        <v>4273</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2452,13 +2450,13 @@
         <v>6</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J80" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K80" s="1" t="n">
-        <v>4228</v>
+        <v>4303</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2466,13 +2464,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J81" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K81" s="1" t="n">
-        <v>4273</v>
+        <v>4124</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2480,13 +2478,13 @@
         <v>6</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J82" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K82" s="1" t="n">
-        <v>4303</v>
+        <v>4185</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2494,13 +2492,13 @@
         <v>6</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J83" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K83" s="1" t="n">
-        <v>4124</v>
+        <v>4063</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2508,13 +2506,13 @@
         <v>6</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J84" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K84" s="1" t="n">
-        <v>4185</v>
+        <v>4274</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2522,13 +2520,13 @@
         <v>6</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J85" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K85" s="1" t="n">
-        <v>4063</v>
+        <v>4095</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2536,13 +2534,13 @@
         <v>6</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J86" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K86" s="1" t="n">
-        <v>4274</v>
+        <v>4193</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2550,13 +2548,13 @@
         <v>6</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J87" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K87" s="1" t="n">
-        <v>4095</v>
+        <v>4003</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2564,13 +2562,13 @@
         <v>6</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J88" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K88" s="1" t="n">
-        <v>4193</v>
+        <v>4229</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2578,13 +2576,13 @@
         <v>6</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J89" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K89" s="1" t="n">
-        <v>4003</v>
+        <v>4064</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2592,13 +2590,13 @@
         <v>6</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J90" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K90" s="1" t="n">
-        <v>4229</v>
+        <v>4230</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,27 +2604,30 @@
         <v>6</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J91" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K91" s="1" t="n">
-        <v>4064</v>
+        <v>4004</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>133</v>
       </c>
       <c r="J92" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K92" s="1" t="n">
-        <v>4230</v>
+        <v>4231</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2640,24 +2641,21 @@
         <v>0</v>
       </c>
       <c r="K93" s="1" t="n">
-        <v>4004</v>
+        <v>4194</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D94" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="J94" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K94" s="1" t="n">
-        <v>4231</v>
+        <v>4065</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2665,13 +2663,13 @@
         <v>6</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J95" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K95" s="1" t="n">
-        <v>4194</v>
+        <v>4304</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2679,13 +2677,13 @@
         <v>6</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J96" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K96" s="1" t="n">
-        <v>4065</v>
+        <v>4134</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2693,13 +2691,13 @@
         <v>6</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J97" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K97" s="1" t="n">
-        <v>4304</v>
+        <v>4066</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2707,13 +2705,13 @@
         <v>6</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J98" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K98" s="1" t="n">
-        <v>4134</v>
+        <v>4195</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2721,13 +2719,13 @@
         <v>6</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J99" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K99" s="1" t="n">
-        <v>4066</v>
+        <v>4049</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2735,27 +2733,30 @@
         <v>6</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J100" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K100" s="1" t="n">
-        <v>4195</v>
+        <v>4161</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B101" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>143</v>
       </c>
       <c r="J101" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K101" s="1" t="n">
-        <v>4049</v>
+        <v>4305</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2769,24 +2770,21 @@
         <v>0</v>
       </c>
       <c r="K102" s="1" t="n">
-        <v>4161</v>
+        <v>4026</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D103" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="J103" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K103" s="1" t="n">
-        <v>4305</v>
+        <v>4005</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2794,27 +2792,30 @@
         <v>6</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J104" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K104" s="1" t="n">
-        <v>4026</v>
+        <v>4196</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B105" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>148</v>
       </c>
       <c r="J105" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K105" s="1" t="n">
-        <v>4005</v>
+        <v>4067</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2828,38 +2829,38 @@
         <v>0</v>
       </c>
       <c r="K106" s="1" t="n">
-        <v>4196</v>
+        <v>4306</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D107" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="J107" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K107" s="1" t="n">
-        <v>4067</v>
+        <v>4027</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B108" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D108" s="1" t="s">
         <v>152</v>
       </c>
       <c r="J108" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K108" s="1" t="n">
-        <v>4306</v>
+        <v>4028</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2873,24 +2874,21 @@
         <v>0</v>
       </c>
       <c r="K109" s="1" t="n">
-        <v>4027</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D110" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="J110" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K110" s="1" t="n">
-        <v>4028</v>
+        <v>4307</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2898,27 +2896,27 @@
         <v>6</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J111" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K111" s="1" t="n">
-        <v>4163</v>
+        <v>4164</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J112" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K112" s="1" t="n">
-        <v>4307</v>
+        <v>4029</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2926,13 +2924,13 @@
         <v>6</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J113" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K113" s="1" t="n">
-        <v>4164</v>
+        <v>4232</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2940,13 +2938,13 @@
         <v>1</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J114" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K114" s="1" t="n">
-        <v>4029</v>
+        <v>4165</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2954,27 +2952,27 @@
         <v>6</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J115" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K115" s="1" t="n">
-        <v>4232</v>
+        <v>4135</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J116" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K116" s="1" t="n">
-        <v>4165</v>
+        <v>4006</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2982,13 +2980,13 @@
         <v>6</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J117" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K117" s="1" t="n">
-        <v>4135</v>
+        <v>4099</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2996,13 +2994,13 @@
         <v>6</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J118" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K118" s="1" t="n">
-        <v>4006</v>
+        <v>4068</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3010,13 +3008,13 @@
         <v>6</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J119" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K119" s="1" t="n">
-        <v>4099</v>
+        <v>4197</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3024,27 +3022,30 @@
         <v>6</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J120" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K120" s="1" t="n">
-        <v>4068</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B121" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D121" s="1" t="s">
         <v>166</v>
       </c>
       <c r="J121" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K121" s="1" t="n">
-        <v>4197</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3058,38 +3059,35 @@
         <v>0</v>
       </c>
       <c r="K122" s="1" t="n">
-        <v>4100</v>
+        <v>4198</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D123" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="J123" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K123" s="1" t="n">
-        <v>4251</v>
+        <v>4186</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J124" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K124" s="1" t="n">
-        <v>4198</v>
+        <v>4007</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3097,27 +3095,27 @@
         <v>6</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J125" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K125" s="1" t="n">
-        <v>4186</v>
+        <v>4199</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J126" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K126" s="1" t="n">
-        <v>4007</v>
+        <v>4136</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3125,13 +3123,13 @@
         <v>6</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J127" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K127" s="1" t="n">
-        <v>4199</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3139,13 +3137,13 @@
         <v>6</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J128" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K128" s="1" t="n">
-        <v>4136</v>
+        <v>4084</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3153,13 +3151,13 @@
         <v>6</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J129" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K129" s="1" t="n">
-        <v>4200</v>
+        <v>4071</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3167,13 +3165,13 @@
         <v>6</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J130" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K130" s="1" t="n">
-        <v>4084</v>
+        <v>4252</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3181,13 +3179,13 @@
         <v>6</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J131" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K131" s="1" t="n">
-        <v>4071</v>
+        <v>4169</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3195,13 +3193,13 @@
         <v>6</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J132" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K132" s="1" t="n">
-        <v>4252</v>
+        <v>4233</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3209,27 +3207,27 @@
         <v>6</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J133" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K133" s="1" t="n">
-        <v>4169</v>
+        <v>4030</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J134" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K134" s="1" t="n">
-        <v>4233</v>
+        <v>4275</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3237,27 +3235,27 @@
         <v>6</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J135" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K135" s="1" t="n">
-        <v>4030</v>
+        <v>4309</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J136" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K136" s="1" t="n">
-        <v>4275</v>
+        <v>4310</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3265,13 +3263,13 @@
         <v>6</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J137" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K137" s="1" t="n">
-        <v>4309</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3279,27 +3277,27 @@
         <v>6</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J138" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K138" s="1" t="n">
-        <v>4310</v>
+        <v>4031</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J139" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K139" s="1" t="n">
-        <v>4276</v>
+        <v>4008</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,27 +3305,27 @@
         <v>6</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J140" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K140" s="1" t="n">
-        <v>4031</v>
+        <v>4170</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J141" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K141" s="1" t="n">
-        <v>4008</v>
+        <v>4311</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3335,27 +3333,30 @@
         <v>6</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J142" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K142" s="1" t="n">
-        <v>4170</v>
+        <v>4137</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
+      </c>
+      <c r="D143" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="J143" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K143" s="1" t="n">
-        <v>4311</v>
+        <v>4312</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3363,30 +3364,27 @@
         <v>6</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J144" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K144" s="1" t="n">
-        <v>4137</v>
+        <v>4201</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="D145" s="4" t="s">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="J145" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K145" s="1" t="n">
-        <v>4312</v>
+        <v>4313</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3394,13 +3392,13 @@
         <v>6</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J146" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K146" s="1" t="n">
-        <v>4201</v>
+        <v>4138</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3408,13 +3406,13 @@
         <v>6</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J147" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K147" s="1" t="n">
-        <v>4313</v>
+        <v>4104</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3422,13 +3420,13 @@
         <v>6</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J148" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K148" s="1" t="n">
-        <v>4138</v>
+        <v>4253</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3436,13 +3434,13 @@
         <v>6</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J149" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K149" s="1" t="n">
-        <v>4104</v>
+        <v>4032</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3450,27 +3448,30 @@
         <v>6</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J150" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K150" s="1" t="n">
-        <v>4253</v>
+        <v>4105</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B151" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D151" s="4" t="s">
         <v>197</v>
       </c>
       <c r="J151" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K151" s="1" t="n">
-        <v>4032</v>
+        <v>4202</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3484,38 +3485,38 @@
         <v>0</v>
       </c>
       <c r="K152" s="1" t="n">
-        <v>4105</v>
+        <v>4314</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D153" s="4" t="s">
-        <v>200</v>
-      </c>
       <c r="J153" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K153" s="1" t="n">
-        <v>4202</v>
+        <v>4033</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B154" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D154" s="1" t="s">
         <v>201</v>
       </c>
       <c r="J154" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K154" s="1" t="n">
-        <v>4314</v>
+        <v>4139</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3529,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="K155" s="1" t="n">
-        <v>4033</v>
+        <v>4234</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3546,38 +3547,38 @@
         <v>0</v>
       </c>
       <c r="K156" s="1" t="n">
-        <v>4139</v>
+        <v>4184</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>205</v>
       </c>
+      <c r="D157" s="1" t="s">
+        <v>206</v>
+      </c>
       <c r="J157" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K157" s="1" t="n">
-        <v>4234</v>
+        <v>4254</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="D158" s="1" t="s">
         <v>207</v>
       </c>
       <c r="J158" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K158" s="1" t="n">
-        <v>4184</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,14 +3588,11 @@
       <c r="B159" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="D159" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="J159" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K159" s="1" t="n">
-        <v>4254</v>
+        <v>4277</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,60 +3600,63 @@
         <v>6</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J160" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K160" s="1" t="n">
-        <v>4106</v>
+        <v>4203</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J161" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K161" s="1" t="n">
-        <v>4277</v>
+        <v>4009</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J162" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K162" s="1" t="n">
-        <v>4203</v>
+        <v>4235</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B163" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D163" s="4" t="s">
         <v>213</v>
       </c>
       <c r="J163" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K163" s="1" t="n">
-        <v>4009</v>
+        <v>4107</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>214</v>
@@ -3664,24 +3665,21 @@
         <v>0</v>
       </c>
       <c r="K164" s="1" t="n">
-        <v>4235</v>
+        <v>4255</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="D165" s="4" t="s">
-        <v>216</v>
-      </c>
       <c r="J165" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K165" s="1" t="n">
-        <v>4107</v>
+        <v>4172</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,13 +3687,13 @@
         <v>6</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J166" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K166" s="1" t="n">
-        <v>4255</v>
+        <v>4279</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,13 +3701,13 @@
         <v>6</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J167" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K167" s="1" t="n">
-        <v>4172</v>
+        <v>4236</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3717,13 +3715,13 @@
         <v>6</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J168" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K168" s="1" t="n">
-        <v>4279</v>
+        <v>4034</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,13 +3729,13 @@
         <v>6</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J169" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K169" s="1" t="n">
-        <v>4236</v>
+        <v>4204</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3745,13 +3743,13 @@
         <v>6</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="J170" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K170" s="1" t="n">
-        <v>4034</v>
+        <v>4035</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,13 +3757,13 @@
         <v>6</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J171" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K171" s="1" t="n">
-        <v>4204</v>
+        <v>4072</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3773,13 +3771,13 @@
         <v>6</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J172" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K172" s="1" t="n">
-        <v>4035</v>
+        <v>4010</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3787,13 +3785,13 @@
         <v>6</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J173" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K173" s="1" t="n">
-        <v>4072</v>
+        <v>4173</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3801,13 +3799,13 @@
         <v>6</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J174" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K174" s="1" t="n">
-        <v>4010</v>
+        <v>4140</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3815,27 +3813,30 @@
         <v>6</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J175" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K175" s="1" t="n">
-        <v>4173</v>
+        <v>4073</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B176" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D176" s="4" t="s">
         <v>227</v>
       </c>
       <c r="J176" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K176" s="1" t="n">
-        <v>4140</v>
+        <v>4256</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3849,24 +3850,21 @@
         <v>0</v>
       </c>
       <c r="K177" s="1" t="n">
-        <v>4073</v>
+        <v>4037</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B178" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="D178" s="4" t="s">
-        <v>230</v>
-      </c>
       <c r="J178" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K178" s="1" t="n">
-        <v>4256</v>
+        <v>4237</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3874,27 +3872,30 @@
         <v>6</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J179" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K179" s="1" t="n">
-        <v>4037</v>
+        <v>4038</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B180" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D180" s="1" t="s">
         <v>232</v>
       </c>
       <c r="J180" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K180" s="1" t="n">
-        <v>4237</v>
+        <v>4074</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,38 +3909,35 @@
         <v>0</v>
       </c>
       <c r="K181" s="1" t="n">
-        <v>4038</v>
+        <v>4175</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B182" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D182" s="1" t="s">
-        <v>235</v>
-      </c>
       <c r="J182" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K182" s="1" t="n">
-        <v>4074</v>
+        <v>4280</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J183" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K183" s="1" t="n">
-        <v>4175</v>
+        <v>4257</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,41 +3945,41 @@
         <v>6</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J184" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K184" s="1" t="n">
-        <v>4280</v>
+        <v>4205</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J185" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K185" s="1" t="n">
-        <v>4257</v>
+        <v>4141</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J186" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K186" s="1" t="n">
-        <v>4205</v>
+        <v>4281</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3989,27 +3987,27 @@
         <v>6</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="J187" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K187" s="1" t="n">
-        <v>4141</v>
+        <v>4039</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J188" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K188" s="1" t="n">
-        <v>4281</v>
+        <v>4110</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,27 +4015,30 @@
         <v>6</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J189" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K189" s="1" t="n">
-        <v>4039</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B190" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D190" s="1" t="s">
         <v>243</v>
       </c>
       <c r="J190" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K190" s="1" t="n">
-        <v>4110</v>
+        <v>4111</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4051,24 +4052,21 @@
         <v>0</v>
       </c>
       <c r="K191" s="1" t="n">
-        <v>4258</v>
+        <v>4282</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="D192" s="1" t="s">
-        <v>246</v>
-      </c>
       <c r="J192" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K192" s="1" t="n">
-        <v>4111</v>
+        <v>4238</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4076,13 +4074,13 @@
         <v>6</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J193" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K193" s="1" t="n">
-        <v>4282</v>
+        <v>4075</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,13 +4088,13 @@
         <v>6</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J194" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K194" s="1" t="n">
-        <v>4238</v>
+        <v>4112</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,13 +4102,13 @@
         <v>6</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J195" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K195" s="1" t="n">
-        <v>4075</v>
+        <v>4206</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,13 +4116,13 @@
         <v>6</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J196" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K196" s="1" t="n">
-        <v>4112</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4132,13 +4130,13 @@
         <v>6</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J197" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K197" s="1" t="n">
-        <v>4206</v>
+        <v>4076</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4146,13 +4144,13 @@
         <v>6</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J198" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K198" s="1" t="n">
-        <v>4283</v>
+        <v>4207</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4160,55 +4158,55 @@
         <v>6</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J199" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K199" s="1" t="n">
-        <v>4076</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J200" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K200" s="1" t="n">
-        <v>4207</v>
+        <v>4142</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J201" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K201" s="1" t="n">
-        <v>4125</v>
+        <v>4143</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J202" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K202" s="1" t="n">
-        <v>4142</v>
+        <v>4318</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4216,13 +4214,13 @@
         <v>1</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J203" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K203" s="1" t="n">
-        <v>4143</v>
+        <v>4144</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4230,27 +4228,27 @@
         <v>6</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J204" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K204" s="1" t="n">
-        <v>4318</v>
+        <v>4259</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J205" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K205" s="1" t="n">
-        <v>4144</v>
+        <v>4176</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4258,13 +4256,13 @@
         <v>6</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J206" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K206" s="1" t="n">
-        <v>4259</v>
+        <v>4208</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4272,13 +4270,13 @@
         <v>6</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J207" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K207" s="1" t="n">
-        <v>4176</v>
+        <v>4209</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4286,13 +4284,13 @@
         <v>6</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J208" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K208" s="1" t="n">
-        <v>4208</v>
+        <v>4319</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4300,13 +4298,13 @@
         <v>6</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J209" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K209" s="1" t="n">
-        <v>4209</v>
+        <v>4239</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4314,13 +4312,13 @@
         <v>6</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J210" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K210" s="1" t="n">
-        <v>4319</v>
+        <v>4177</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4328,27 +4326,27 @@
         <v>6</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J211" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K211" s="1" t="n">
-        <v>4239</v>
+        <v>4040</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J212" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K212" s="1" t="n">
-        <v>4177</v>
+        <v>4284</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4356,27 +4354,27 @@
         <v>6</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J213" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K213" s="1" t="n">
-        <v>4040</v>
+        <v>4210</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J214" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K214" s="1" t="n">
-        <v>4284</v>
+        <v>4260</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4384,13 +4382,13 @@
         <v>6</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J215" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K215" s="1" t="n">
-        <v>4210</v>
+        <v>4041</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4398,41 +4396,41 @@
         <v>6</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J216" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K216" s="1" t="n">
-        <v>4260</v>
+        <v>4285</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J217" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K217" s="1" t="n">
-        <v>4041</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J218" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K218" s="1" t="n">
-        <v>4285</v>
+        <v>4077</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4440,44 +4438,44 @@
         <v>1</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
+      </c>
+      <c r="D219" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="J219" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K219" s="1" t="n">
-        <v>4012</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J220" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K220" s="1" t="n">
-        <v>4077</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="D221" s="1" t="s">
-        <v>146</v>
+        <v>274</v>
       </c>
       <c r="J221" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K221" s="1" t="n">
-        <v>4320</v>
+        <v>4117</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4485,13 +4483,13 @@
         <v>6</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J222" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K222" s="1" t="n">
-        <v>4145</v>
+        <v>4286</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4499,13 +4497,13 @@
         <v>6</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J223" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K223" s="1" t="n">
-        <v>4117</v>
+        <v>4078</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4513,13 +4511,13 @@
         <v>6</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J224" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K224" s="1" t="n">
-        <v>4286</v>
+        <v>4013</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4527,27 +4525,27 @@
         <v>6</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J225" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K225" s="1" t="n">
-        <v>4078</v>
+        <v>4146</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J226" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K226" s="1" t="n">
-        <v>4013</v>
+        <v>4079</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4555,27 +4553,27 @@
         <v>6</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J227" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K227" s="1" t="n">
-        <v>4146</v>
+        <v>4044</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J228" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K228" s="1" t="n">
-        <v>4079</v>
+        <v>4120</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4583,13 +4581,13 @@
         <v>6</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J229" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K229" s="1" t="n">
-        <v>4044</v>
+        <v>4121</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4597,13 +4595,13 @@
         <v>6</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J230" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K230" s="1" t="n">
-        <v>4120</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4611,13 +4609,13 @@
         <v>6</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J231" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K231" s="1" t="n">
-        <v>4121</v>
+        <v>4122</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4625,27 +4623,30 @@
         <v>6</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J232" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K232" s="1" t="n">
-        <v>4080</v>
+        <v>4287</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B233" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="D233" s="4" t="s">
         <v>287</v>
       </c>
       <c r="J233" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K233" s="1" t="n">
-        <v>4122</v>
+        <v>4261</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4659,24 +4660,21 @@
         <v>0</v>
       </c>
       <c r="K234" s="1" t="n">
-        <v>4287</v>
+        <v>4240</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B235" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="D235" s="4" t="s">
-        <v>290</v>
-      </c>
       <c r="J235" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K235" s="1" t="n">
-        <v>4261</v>
+        <v>4262</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4684,13 +4682,13 @@
         <v>6</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J236" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K236" s="1" t="n">
-        <v>4240</v>
+        <v>4045</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4698,27 +4696,27 @@
         <v>6</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J237" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K237" s="1" t="n">
-        <v>4262</v>
+        <v>4081</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J238" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K238" s="1" t="n">
-        <v>4045</v>
+        <v>4288</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4726,27 +4724,27 @@
         <v>6</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J239" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K239" s="1" t="n">
-        <v>4081</v>
+        <v>4123</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J240" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K240" s="1" t="n">
-        <v>4288</v>
+        <v>4181</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4754,13 +4752,13 @@
         <v>6</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J241" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K241" s="1" t="n">
-        <v>4123</v>
+        <v>4082</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4768,13 +4766,13 @@
         <v>6</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J242" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K242" s="1" t="n">
-        <v>4181</v>
+        <v>4046</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4782,27 +4780,30 @@
         <v>6</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J243" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K243" s="1" t="n">
-        <v>4082</v>
+        <v>4182</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B244" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D244" s="4" t="s">
         <v>299</v>
       </c>
       <c r="J244" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K244" s="1" t="n">
-        <v>4046</v>
+        <v>4047</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4816,24 +4817,21 @@
         <v>0</v>
       </c>
       <c r="K245" s="1" t="n">
-        <v>4182</v>
+        <v>4048</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B246" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="D246" s="4" t="s">
-        <v>302</v>
-      </c>
       <c r="J246" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K246" s="1" t="n">
-        <v>4047</v>
+        <v>4183</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4841,13 +4839,13 @@
         <v>6</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J247" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K247" s="1" t="n">
-        <v>4048</v>
+        <v>4263</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4855,13 +4853,13 @@
         <v>6</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J248" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K248" s="1" t="n">
-        <v>4183</v>
+        <v>4147</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4869,13 +4867,13 @@
         <v>6</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J249" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K249" s="1" t="n">
-        <v>4263</v>
+        <v>4289</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4883,13 +4881,13 @@
         <v>6</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J250" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K250" s="1" t="n">
-        <v>4147</v>
+        <v>4083</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4897,163 +4895,163 @@
         <v>6</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J251" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K251" s="1" t="n">
-        <v>4289</v>
+        <v>4324</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B252" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D252" s="1" t="s">
         <v>308</v>
       </c>
       <c r="J252" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K252" s="1" t="n">
-        <v>4083</v>
-      </c>
-    </row>
-    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4264</v>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B253" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B253" s="8" t="s">
         <v>309</v>
       </c>
+      <c r="C253" s="8"/>
       <c r="J253" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K253" s="1" t="n">
-        <v>4324</v>
-      </c>
-    </row>
-    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4323</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B254" s="1" t="s">
+      <c r="B254" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="D254" s="1" t="s">
-        <v>311</v>
-      </c>
+      <c r="C254" s="8"/>
       <c r="J254" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K254" s="1" t="n">
-        <v>4264</v>
+        <v>4094</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B255" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="C255" s="7"/>
+      <c r="B255" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="C255" s="8"/>
       <c r="J255" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K255" s="1" t="n">
-        <v>4323</v>
+        <v>4308</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B256" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="C256" s="7"/>
+      <c r="B256" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="C256" s="8"/>
       <c r="J256" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K256" s="1" t="n">
-        <v>4094</v>
+        <v>4317</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B257" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="C257" s="7"/>
+      <c r="B257" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="C257" s="8"/>
       <c r="J257" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K257" s="1" t="n">
-        <v>4308</v>
+        <v>4113</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B258" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="C258" s="7"/>
+      <c r="B258" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="C258" s="8"/>
       <c r="J258" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K258" s="1" t="n">
-        <v>4317</v>
+        <v>4042</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B259" s="7" t="s">
+      <c r="B259" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="C259" s="8"/>
+      <c r="J259" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K259" s="1" t="n">
+        <v>4179</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B260" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C259" s="7"/>
-      <c r="J259" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K259" s="1" t="n">
-        <v>4113</v>
-      </c>
-    </row>
-    <row r="260" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B260" s="7" t="s">
+      <c r="J260" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K260" s="1" t="n">
+        <v>4114</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B261" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="C260" s="7"/>
-      <c r="J260" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K260" s="1" t="n">
-        <v>4042</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B261" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="C261" s="7"/>
       <c r="J261" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K261" s="1" t="n">
-        <v>4179</v>
+        <v>4321</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5061,63 +5059,37 @@
         <v>1</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J262" s="1" t="n">
         <v>1</v>
       </c>
       <c r="K262" s="1" t="n">
-        <v>4114</v>
-      </c>
-    </row>
-    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A263" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B263" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="J263" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K263" s="1" t="n">
-        <v>4321</v>
-      </c>
-    </row>
-    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A264" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B264" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="J264" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K264" s="1" t="n">
         <v>4133</v>
       </c>
     </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:K264"/>
+  <autoFilter ref="A1:K262"/>
   <mergeCells count="1">
     <mergeCell ref="C42:D42"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="baubewilligungen@ag.ch"/>
-    <hyperlink ref="D145" r:id="rId2" display="bauverwaltung@unterendingen.ch"/>
-    <hyperlink ref="D153" r:id="rId3" display="gemeinde@meisterschwanden.ch"/>
-    <hyperlink ref="D165" r:id="rId4" display="gemeindekanzlei@muelligen.ch"/>
-    <hyperlink ref="D178" r:id="rId5" display="bauverwaltung@obermumpf.ch"/>
-    <hyperlink ref="D235" r:id="rId6" display="bauverwaltung@wallbach.ch"/>
-    <hyperlink ref="D246" r:id="rId7" display="bauverwaltung@wuerenlingen.ch"/>
+    <hyperlink ref="D143" r:id="rId2" display="bauverwaltung@unterendingen.ch"/>
+    <hyperlink ref="D151" r:id="rId3" display="gemeinde@meisterschwanden.ch"/>
+    <hyperlink ref="D163" r:id="rId4" display="gemeindekanzlei@muelligen.ch"/>
+    <hyperlink ref="D176" r:id="rId5" display="bauverwaltung@obermumpf.ch"/>
+    <hyperlink ref="D233" r:id="rId6" display="bauverwaltung@wallbach.ch"/>
+    <hyperlink ref="D244" r:id="rId7" display="bauverwaltung@wuerenlingen.ch"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
   <drawing r:id="rId8"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(ag): add services sbb and procap
</commit_message>
<xml_diff>
--- a/django/kt_ag/import/Services_AG.xlsx
+++ b/django/kt_ag/import/Services_AG.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="320">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">SBB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sbb</t>
   </si>
   <si>
     <t xml:space="preserve">Technisches Inspektorat des Schweizerischen Gasfachs (TISG)</t>
@@ -2039,6 +2042,9 @@
       <c r="B52" s="1" t="s">
         <v>84</v>
       </c>
+      <c r="C52" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="J52" s="1" t="n">
         <v>0</v>
       </c>
@@ -2048,7 +2054,7 @@
         <v>4</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J53" s="1" t="n">
         <v>0</v>
@@ -2059,22 +2065,22 @@
         <v>4</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E54" s="1" t="n">
         <v>4600</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H54" s="1" t="n">
         <v>622068850</v>
@@ -2088,10 +2094,10 @@
         <v>5</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J55" s="1" t="n">
         <v>0</v>
@@ -2116,10 +2122,10 @@
         <v>1</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J57" s="1" t="n">
         <v>0</v>
@@ -2133,10 +2139,10 @@
         <v>6</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J58" s="1" t="n">
         <v>0</v>
@@ -2150,7 +2156,7 @@
         <v>6</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J59" s="1" t="n">
         <v>0</v>
@@ -2164,7 +2170,7 @@
         <v>6</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J60" s="1" t="n">
         <v>0</v>
@@ -2178,10 +2184,10 @@
         <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J61" s="1" t="n">
         <v>0</v>
@@ -2195,7 +2201,7 @@
         <v>6</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J62" s="1" t="n">
         <v>0</v>
@@ -2209,7 +2215,7 @@
         <v>6</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J63" s="1" t="n">
         <v>0</v>
@@ -2223,7 +2229,7 @@
         <v>6</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J64" s="1" t="n">
         <v>0</v>
@@ -2237,7 +2243,7 @@
         <v>6</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J65" s="1" t="n">
         <v>0</v>
@@ -2251,7 +2257,7 @@
         <v>6</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J66" s="1" t="n">
         <v>0</v>
@@ -2265,7 +2271,7 @@
         <v>6</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J67" s="1" t="n">
         <v>0</v>
@@ -2279,7 +2285,7 @@
         <v>6</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J68" s="1" t="n">
         <v>0</v>
@@ -2293,7 +2299,7 @@
         <v>6</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J69" s="1" t="n">
         <v>0</v>
@@ -2307,7 +2313,7 @@
         <v>6</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J70" s="1" t="n">
         <v>0</v>
@@ -2321,7 +2327,7 @@
         <v>6</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J71" s="1" t="n">
         <v>0</v>
@@ -2335,10 +2341,10 @@
         <v>1</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J72" s="1" t="n">
         <v>0</v>
@@ -2352,7 +2358,7 @@
         <v>6</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J73" s="1" t="n">
         <v>0</v>
@@ -2366,7 +2372,7 @@
         <v>6</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J74" s="1" t="n">
         <v>0</v>
@@ -2380,7 +2386,7 @@
         <v>6</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J75" s="1" t="n">
         <v>0</v>
@@ -2394,7 +2400,7 @@
         <v>6</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J76" s="1" t="n">
         <v>0</v>
@@ -2408,7 +2414,7 @@
         <v>6</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J77" s="1" t="n">
         <v>0</v>
@@ -2422,7 +2428,7 @@
         <v>6</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J78" s="1" t="n">
         <v>0</v>
@@ -2436,7 +2442,7 @@
         <v>6</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J79" s="1" t="n">
         <v>0</v>
@@ -2450,7 +2456,7 @@
         <v>6</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J80" s="1" t="n">
         <v>0</v>
@@ -2464,7 +2470,7 @@
         <v>6</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J81" s="1" t="n">
         <v>0</v>
@@ -2478,7 +2484,7 @@
         <v>6</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J82" s="1" t="n">
         <v>0</v>
@@ -2492,7 +2498,7 @@
         <v>6</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J83" s="1" t="n">
         <v>0</v>
@@ -2506,7 +2512,7 @@
         <v>6</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J84" s="1" t="n">
         <v>0</v>
@@ -2520,7 +2526,7 @@
         <v>6</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J85" s="1" t="n">
         <v>0</v>
@@ -2534,7 +2540,7 @@
         <v>6</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J86" s="1" t="n">
         <v>0</v>
@@ -2548,7 +2554,7 @@
         <v>6</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J87" s="1" t="n">
         <v>0</v>
@@ -2562,7 +2568,7 @@
         <v>6</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J88" s="1" t="n">
         <v>0</v>
@@ -2576,7 +2582,7 @@
         <v>6</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J89" s="1" t="n">
         <v>0</v>
@@ -2590,7 +2596,7 @@
         <v>6</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J90" s="1" t="n">
         <v>0</v>
@@ -2604,7 +2610,7 @@
         <v>6</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J91" s="1" t="n">
         <v>0</v>
@@ -2618,10 +2624,10 @@
         <v>1</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J92" s="1" t="n">
         <v>0</v>
@@ -2635,7 +2641,7 @@
         <v>6</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J93" s="1" t="n">
         <v>0</v>
@@ -2649,7 +2655,7 @@
         <v>6</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J94" s="1" t="n">
         <v>0</v>
@@ -2663,7 +2669,7 @@
         <v>6</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J95" s="1" t="n">
         <v>0</v>
@@ -2677,7 +2683,7 @@
         <v>6</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J96" s="1" t="n">
         <v>0</v>
@@ -2691,7 +2697,7 @@
         <v>6</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J97" s="1" t="n">
         <v>0</v>
@@ -2705,7 +2711,7 @@
         <v>6</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J98" s="1" t="n">
         <v>0</v>
@@ -2719,7 +2725,7 @@
         <v>6</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J99" s="1" t="n">
         <v>0</v>
@@ -2733,7 +2739,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J100" s="1" t="n">
         <v>0</v>
@@ -2747,10 +2753,10 @@
         <v>1</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J101" s="1" t="n">
         <v>0</v>
@@ -2764,7 +2770,7 @@
         <v>6</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J102" s="1" t="n">
         <v>0</v>
@@ -2778,7 +2784,7 @@
         <v>6</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J103" s="1" t="n">
         <v>0</v>
@@ -2792,7 +2798,7 @@
         <v>6</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J104" s="1" t="n">
         <v>0</v>
@@ -2806,10 +2812,10 @@
         <v>1</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J105" s="1" t="n">
         <v>0</v>
@@ -2823,7 +2829,7 @@
         <v>6</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J106" s="1" t="n">
         <v>0</v>
@@ -2837,7 +2843,7 @@
         <v>6</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J107" s="1" t="n">
         <v>0</v>
@@ -2851,10 +2857,10 @@
         <v>1</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J108" s="1" t="n">
         <v>0</v>
@@ -2868,7 +2874,7 @@
         <v>6</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J109" s="1" t="n">
         <v>0</v>
@@ -2882,7 +2888,7 @@
         <v>6</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J110" s="1" t="n">
         <v>0</v>
@@ -2896,7 +2902,7 @@
         <v>6</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J111" s="1" t="n">
         <v>0</v>
@@ -2910,7 +2916,7 @@
         <v>1</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J112" s="1" t="n">
         <v>0</v>
@@ -2924,7 +2930,7 @@
         <v>6</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J113" s="1" t="n">
         <v>0</v>
@@ -2938,7 +2944,7 @@
         <v>1</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J114" s="1" t="n">
         <v>0</v>
@@ -2952,7 +2958,7 @@
         <v>6</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J115" s="1" t="n">
         <v>0</v>
@@ -2966,7 +2972,7 @@
         <v>6</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J116" s="1" t="n">
         <v>0</v>
@@ -2980,7 +2986,7 @@
         <v>6</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J117" s="1" t="n">
         <v>0</v>
@@ -2994,7 +3000,7 @@
         <v>6</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J118" s="1" t="n">
         <v>0</v>
@@ -3008,7 +3014,7 @@
         <v>6</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J119" s="1" t="n">
         <v>0</v>
@@ -3022,7 +3028,7 @@
         <v>6</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J120" s="1" t="n">
         <v>0</v>
@@ -3036,10 +3042,10 @@
         <v>1</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J121" s="1" t="n">
         <v>0</v>
@@ -3053,7 +3059,7 @@
         <v>6</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J122" s="1" t="n">
         <v>0</v>
@@ -3067,7 +3073,7 @@
         <v>6</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J123" s="1" t="n">
         <v>0</v>
@@ -3081,7 +3087,7 @@
         <v>1</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J124" s="1" t="n">
         <v>0</v>
@@ -3095,7 +3101,7 @@
         <v>6</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J125" s="1" t="n">
         <v>0</v>
@@ -3109,7 +3115,7 @@
         <v>6</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J126" s="1" t="n">
         <v>0</v>
@@ -3123,7 +3129,7 @@
         <v>6</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J127" s="1" t="n">
         <v>0</v>
@@ -3137,7 +3143,7 @@
         <v>6</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J128" s="1" t="n">
         <v>0</v>
@@ -3151,7 +3157,7 @@
         <v>6</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J129" s="1" t="n">
         <v>0</v>
@@ -3165,7 +3171,7 @@
         <v>6</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J130" s="1" t="n">
         <v>0</v>
@@ -3179,7 +3185,7 @@
         <v>6</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J131" s="1" t="n">
         <v>0</v>
@@ -3193,7 +3199,7 @@
         <v>6</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J132" s="1" t="n">
         <v>0</v>
@@ -3207,7 +3213,7 @@
         <v>6</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J133" s="1" t="n">
         <v>0</v>
@@ -3221,7 +3227,7 @@
         <v>1</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J134" s="1" t="n">
         <v>0</v>
@@ -3235,7 +3241,7 @@
         <v>6</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J135" s="1" t="n">
         <v>0</v>
@@ -3249,7 +3255,7 @@
         <v>6</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J136" s="1" t="n">
         <v>0</v>
@@ -3263,7 +3269,7 @@
         <v>6</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J137" s="1" t="n">
         <v>0</v>
@@ -3277,7 +3283,7 @@
         <v>6</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J138" s="1" t="n">
         <v>0</v>
@@ -3291,7 +3297,7 @@
         <v>1</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J139" s="1" t="n">
         <v>0</v>
@@ -3305,7 +3311,7 @@
         <v>6</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J140" s="1" t="n">
         <v>0</v>
@@ -3319,7 +3325,7 @@
         <v>6</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J141" s="1" t="n">
         <v>0</v>
@@ -3333,7 +3339,7 @@
         <v>6</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J142" s="1" t="n">
         <v>0</v>
@@ -3347,10 +3353,10 @@
         <v>1</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J143" s="1" t="n">
         <v>0</v>
@@ -3364,7 +3370,7 @@
         <v>6</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J144" s="1" t="n">
         <v>0</v>
@@ -3378,7 +3384,7 @@
         <v>6</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J145" s="1" t="n">
         <v>0</v>
@@ -3392,7 +3398,7 @@
         <v>6</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J146" s="1" t="n">
         <v>0</v>
@@ -3406,7 +3412,7 @@
         <v>6</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J147" s="1" t="n">
         <v>0</v>
@@ -3420,7 +3426,7 @@
         <v>6</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J148" s="1" t="n">
         <v>0</v>
@@ -3434,7 +3440,7 @@
         <v>6</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J149" s="1" t="n">
         <v>0</v>
@@ -3448,7 +3454,7 @@
         <v>6</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J150" s="1" t="n">
         <v>0</v>
@@ -3462,10 +3468,10 @@
         <v>1</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J151" s="1" t="n">
         <v>0</v>
@@ -3479,7 +3485,7 @@
         <v>6</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J152" s="1" t="n">
         <v>0</v>
@@ -3493,7 +3499,7 @@
         <v>6</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J153" s="1" t="n">
         <v>0</v>
@@ -3507,10 +3513,10 @@
         <v>1</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J154" s="1" t="n">
         <v>0</v>
@@ -3524,7 +3530,7 @@
         <v>6</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J155" s="1" t="n">
         <v>0</v>
@@ -3538,10 +3544,10 @@
         <v>1</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J156" s="1" t="n">
         <v>0</v>
@@ -3555,10 +3561,10 @@
         <v>1</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J157" s="1" t="n">
         <v>0</v>
@@ -3572,7 +3578,7 @@
         <v>6</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J158" s="1" t="n">
         <v>0</v>
@@ -3586,7 +3592,7 @@
         <v>1</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J159" s="1" t="n">
         <v>0</v>
@@ -3600,7 +3606,7 @@
         <v>6</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J160" s="1" t="n">
         <v>0</v>
@@ -3614,7 +3620,7 @@
         <v>6</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J161" s="1" t="n">
         <v>0</v>
@@ -3628,7 +3634,7 @@
         <v>1</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J162" s="1" t="n">
         <v>0</v>
@@ -3642,10 +3648,10 @@
         <v>1</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J163" s="1" t="n">
         <v>0</v>
@@ -3659,7 +3665,7 @@
         <v>6</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J164" s="1" t="n">
         <v>0</v>
@@ -3673,7 +3679,7 @@
         <v>6</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J165" s="1" t="n">
         <v>0</v>
@@ -3687,7 +3693,7 @@
         <v>6</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J166" s="1" t="n">
         <v>0</v>
@@ -3701,7 +3707,7 @@
         <v>6</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J167" s="1" t="n">
         <v>0</v>
@@ -3715,7 +3721,7 @@
         <v>6</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J168" s="1" t="n">
         <v>0</v>
@@ -3729,7 +3735,7 @@
         <v>6</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J169" s="1" t="n">
         <v>0</v>
@@ -3743,7 +3749,7 @@
         <v>6</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J170" s="1" t="n">
         <v>0</v>
@@ -3757,7 +3763,7 @@
         <v>6</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J171" s="1" t="n">
         <v>0</v>
@@ -3771,7 +3777,7 @@
         <v>6</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J172" s="1" t="n">
         <v>0</v>
@@ -3785,7 +3791,7 @@
         <v>6</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J173" s="1" t="n">
         <v>0</v>
@@ -3799,7 +3805,7 @@
         <v>6</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J174" s="1" t="n">
         <v>0</v>
@@ -3813,7 +3819,7 @@
         <v>6</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J175" s="1" t="n">
         <v>0</v>
@@ -3827,10 +3833,10 @@
         <v>1</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D176" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J176" s="1" t="n">
         <v>0</v>
@@ -3844,7 +3850,7 @@
         <v>6</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J177" s="1" t="n">
         <v>0</v>
@@ -3858,7 +3864,7 @@
         <v>6</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J178" s="1" t="n">
         <v>0</v>
@@ -3872,7 +3878,7 @@
         <v>6</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J179" s="1" t="n">
         <v>0</v>
@@ -3886,10 +3892,10 @@
         <v>1</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D180" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J180" s="1" t="n">
         <v>0</v>
@@ -3903,7 +3909,7 @@
         <v>6</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J181" s="1" t="n">
         <v>0</v>
@@ -3917,7 +3923,7 @@
         <v>6</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J182" s="1" t="n">
         <v>0</v>
@@ -3931,7 +3937,7 @@
         <v>1</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J183" s="1" t="n">
         <v>0</v>
@@ -3945,7 +3951,7 @@
         <v>6</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J184" s="1" t="n">
         <v>0</v>
@@ -3959,7 +3965,7 @@
         <v>6</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J185" s="1" t="n">
         <v>0</v>
@@ -3973,7 +3979,7 @@
         <v>1</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J186" s="1" t="n">
         <v>0</v>
@@ -3987,7 +3993,7 @@
         <v>6</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J187" s="1" t="n">
         <v>0</v>
@@ -4001,7 +4007,7 @@
         <v>6</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J188" s="1" t="n">
         <v>0</v>
@@ -4015,7 +4021,7 @@
         <v>6</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J189" s="1" t="n">
         <v>0</v>
@@ -4029,10 +4035,10 @@
         <v>1</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D190" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J190" s="1" t="n">
         <v>0</v>
@@ -4046,7 +4052,7 @@
         <v>6</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J191" s="1" t="n">
         <v>0</v>
@@ -4060,7 +4066,7 @@
         <v>6</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J192" s="1" t="n">
         <v>0</v>
@@ -4074,7 +4080,7 @@
         <v>6</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J193" s="1" t="n">
         <v>0</v>
@@ -4088,7 +4094,7 @@
         <v>6</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J194" s="1" t="n">
         <v>0</v>
@@ -4102,7 +4108,7 @@
         <v>6</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J195" s="1" t="n">
         <v>0</v>
@@ -4116,7 +4122,7 @@
         <v>6</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J196" s="1" t="n">
         <v>0</v>
@@ -4130,7 +4136,7 @@
         <v>6</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J197" s="1" t="n">
         <v>0</v>
@@ -4144,7 +4150,7 @@
         <v>6</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J198" s="1" t="n">
         <v>0</v>
@@ -4158,7 +4164,7 @@
         <v>6</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J199" s="1" t="n">
         <v>0</v>
@@ -4172,7 +4178,7 @@
         <v>1</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J200" s="1" t="n">
         <v>0</v>
@@ -4186,7 +4192,7 @@
         <v>1</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J201" s="1" t="n">
         <v>0</v>
@@ -4200,7 +4206,7 @@
         <v>6</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J202" s="1" t="n">
         <v>0</v>
@@ -4214,7 +4220,7 @@
         <v>1</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J203" s="1" t="n">
         <v>0</v>
@@ -4228,7 +4234,7 @@
         <v>6</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J204" s="1" t="n">
         <v>0</v>
@@ -4242,7 +4248,7 @@
         <v>6</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J205" s="1" t="n">
         <v>0</v>
@@ -4256,7 +4262,7 @@
         <v>6</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J206" s="1" t="n">
         <v>0</v>
@@ -4270,7 +4276,7 @@
         <v>6</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J207" s="1" t="n">
         <v>0</v>
@@ -4284,7 +4290,7 @@
         <v>6</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J208" s="1" t="n">
         <v>0</v>
@@ -4298,7 +4304,7 @@
         <v>6</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J209" s="1" t="n">
         <v>0</v>
@@ -4312,7 +4318,7 @@
         <v>6</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J210" s="1" t="n">
         <v>0</v>
@@ -4326,7 +4332,7 @@
         <v>6</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J211" s="1" t="n">
         <v>0</v>
@@ -4340,7 +4346,7 @@
         <v>1</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J212" s="1" t="n">
         <v>0</v>
@@ -4354,7 +4360,7 @@
         <v>6</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J213" s="1" t="n">
         <v>0</v>
@@ -4368,7 +4374,7 @@
         <v>6</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J214" s="1" t="n">
         <v>0</v>
@@ -4382,7 +4388,7 @@
         <v>6</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J215" s="1" t="n">
         <v>0</v>
@@ -4396,7 +4402,7 @@
         <v>6</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J216" s="1" t="n">
         <v>0</v>
@@ -4410,7 +4416,7 @@
         <v>1</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J217" s="1" t="n">
         <v>0</v>
@@ -4424,7 +4430,7 @@
         <v>1</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="J218" s="1" t="n">
         <v>0</v>
@@ -4438,10 +4444,10 @@
         <v>1</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D219" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J219" s="1" t="n">
         <v>0</v>
@@ -4455,7 +4461,7 @@
         <v>6</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J220" s="1" t="n">
         <v>0</v>
@@ -4469,7 +4475,7 @@
         <v>6</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J221" s="1" t="n">
         <v>0</v>
@@ -4483,7 +4489,7 @@
         <v>6</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J222" s="1" t="n">
         <v>0</v>
@@ -4497,7 +4503,7 @@
         <v>6</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J223" s="1" t="n">
         <v>0</v>
@@ -4511,7 +4517,7 @@
         <v>6</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J224" s="1" t="n">
         <v>0</v>
@@ -4525,7 +4531,7 @@
         <v>6</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J225" s="1" t="n">
         <v>0</v>
@@ -4539,7 +4545,7 @@
         <v>1</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J226" s="1" t="n">
         <v>0</v>
@@ -4553,7 +4559,7 @@
         <v>6</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J227" s="1" t="n">
         <v>0</v>
@@ -4567,7 +4573,7 @@
         <v>6</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J228" s="1" t="n">
         <v>0</v>
@@ -4581,7 +4587,7 @@
         <v>6</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J229" s="1" t="n">
         <v>0</v>
@@ -4595,7 +4601,7 @@
         <v>6</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J230" s="1" t="n">
         <v>0</v>
@@ -4609,7 +4615,7 @@
         <v>6</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J231" s="1" t="n">
         <v>0</v>
@@ -4623,7 +4629,7 @@
         <v>6</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J232" s="1" t="n">
         <v>0</v>
@@ -4637,10 +4643,10 @@
         <v>1</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D233" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J233" s="1" t="n">
         <v>0</v>
@@ -4654,7 +4660,7 @@
         <v>6</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J234" s="1" t="n">
         <v>0</v>
@@ -4668,7 +4674,7 @@
         <v>6</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J235" s="1" t="n">
         <v>0</v>
@@ -4682,7 +4688,7 @@
         <v>6</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J236" s="1" t="n">
         <v>0</v>
@@ -4696,7 +4702,7 @@
         <v>6</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J237" s="1" t="n">
         <v>0</v>
@@ -4710,7 +4716,7 @@
         <v>1</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J238" s="1" t="n">
         <v>0</v>
@@ -4724,7 +4730,7 @@
         <v>6</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J239" s="1" t="n">
         <v>0</v>
@@ -4738,7 +4744,7 @@
         <v>6</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J240" s="1" t="n">
         <v>0</v>
@@ -4752,7 +4758,7 @@
         <v>6</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J241" s="1" t="n">
         <v>0</v>
@@ -4766,7 +4772,7 @@
         <v>6</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J242" s="1" t="n">
         <v>0</v>
@@ -4780,7 +4786,7 @@
         <v>6</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J243" s="1" t="n">
         <v>0</v>
@@ -4794,10 +4800,10 @@
         <v>1</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D244" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J244" s="1" t="n">
         <v>0</v>
@@ -4811,7 +4817,7 @@
         <v>6</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J245" s="1" t="n">
         <v>0</v>
@@ -4825,7 +4831,7 @@
         <v>6</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J246" s="1" t="n">
         <v>0</v>
@@ -4839,7 +4845,7 @@
         <v>6</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J247" s="1" t="n">
         <v>0</v>
@@ -4853,7 +4859,7 @@
         <v>6</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J248" s="1" t="n">
         <v>0</v>
@@ -4867,7 +4873,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J249" s="1" t="n">
         <v>0</v>
@@ -4881,7 +4887,7 @@
         <v>6</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J250" s="1" t="n">
         <v>0</v>
@@ -4895,7 +4901,7 @@
         <v>6</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J251" s="1" t="n">
         <v>0</v>
@@ -4909,10 +4915,10 @@
         <v>1</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D252" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J252" s="1" t="n">
         <v>0</v>
@@ -4926,7 +4932,7 @@
         <v>1</v>
       </c>
       <c r="B253" s="8" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C253" s="8"/>
       <c r="J253" s="1" t="n">
@@ -4941,7 +4947,7 @@
         <v>1</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C254" s="8"/>
       <c r="J254" s="1" t="n">
@@ -4956,7 +4962,7 @@
         <v>1</v>
       </c>
       <c r="B255" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C255" s="8"/>
       <c r="J255" s="1" t="n">
@@ -4971,7 +4977,7 @@
         <v>1</v>
       </c>
       <c r="B256" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C256" s="8"/>
       <c r="J256" s="1" t="n">
@@ -4986,7 +4992,7 @@
         <v>1</v>
       </c>
       <c r="B257" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C257" s="8"/>
       <c r="J257" s="1" t="n">
@@ -5001,7 +5007,7 @@
         <v>1</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C258" s="8"/>
       <c r="J258" s="1" t="n">
@@ -5016,7 +5022,7 @@
         <v>1</v>
       </c>
       <c r="B259" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C259" s="8"/>
       <c r="J259" s="1" t="n">
@@ -5031,7 +5037,7 @@
         <v>1</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="J260" s="1" t="n">
         <v>1</v>
@@ -5045,7 +5051,7 @@
         <v>1</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J261" s="1" t="n">
         <v>1</v>
@@ -5059,7 +5065,7 @@
         <v>1</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J262" s="1" t="n">
         <v>1</v>

</xml_diff>